<commit_message>
Refactor Code.gs by AI to improve code quality
</commit_message>
<xml_diff>
--- a/Deal-Watch-Template.xlsx
+++ b/Deal-Watch-Template.xlsx
@@ -7,14 +7,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Home" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runs" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Rules'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Log'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Runs'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Rules'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Log'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Runs'!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,6 +431,72 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Deal Watch — manage everything from Telegram.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Rules / Log / Runs stay hidden; the watcher manages them. Do not edit them by hand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Get started:</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1. In this Sheet: Deal Watch &gt; Setup (paste the bot token, deploy once, paste the /exec URL).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2. In Telegram: open your bot and send /start &lt;token&gt; (single-use).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>3. Add rules in Telegram. Keep this Home sheet visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Help: see README.md in the GitHub repo. Do not delete sheets.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -479,7 +546,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -534,7 +601,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>